<commit_message>
Fix NPER sign bug; add visual preview renders
- Remove stray minus from NPER: -NPER(...) → NPER(...)
  Credit Card now shows +29.8 months (was -29.8)
- Total Interest now positive (Credit Card ≈ $968)
- Add render_previews.py: matplotlib renders of all 6 key tabs to PNG + PDF
- 30 tabs, 4789 formulas, 0 formula errors

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ck3NhBqUmzVxAWdcLovRA6
</commit_message>
<xml_diff>
--- a/The Ultimate Budget.xlsx
+++ b/The Ultimate Budget.xlsx
@@ -247,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -369,6 +369,8 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="14" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -10331,7 +10333,7 @@
         <v>150</v>
       </c>
       <c r="G3" s="61">
-        <f>IF(OR(D3=0,F3=0),IF(F3=0,0,CEILING(C3/F3,1)),IFERROR(-NPER(D3/100/12,-F3,C3),0))</f>
+        <f>IF(OR(D3=0,F3=0),IF(F3=0,0,CEILING(C3/F3,1)),IFERROR(NPER(D3/100/12,-F3,C3),0))</f>
         <v/>
       </c>
       <c r="H3" s="48">
@@ -10365,7 +10367,7 @@
         <v>250</v>
       </c>
       <c r="G4" s="61">
-        <f>IF(OR(D4=0,F4=0),IF(F4=0,0,CEILING(C4/F4,1)),IFERROR(-NPER(D4/100/12,-F4,C4),0))</f>
+        <f>IF(OR(D4=0,F4=0),IF(F4=0,0,CEILING(C4/F4,1)),IFERROR(NPER(D4/100/12,-F4,C4),0))</f>
         <v/>
       </c>
       <c r="H4" s="48">
@@ -10399,7 +10401,7 @@
         <v>300</v>
       </c>
       <c r="G5" s="61">
-        <f>IF(OR(D5=0,F5=0),IF(F5=0,0,CEILING(C5/F5,1)),IFERROR(-NPER(D5/100/12,-F5,C5),0))</f>
+        <f>IF(OR(D5=0,F5=0),IF(F5=0,0,CEILING(C5/F5,1)),IFERROR(NPER(D5/100/12,-F5,C5),0))</f>
         <v/>
       </c>
       <c r="H5" s="48">
@@ -10433,7 +10435,7 @@
         <v>150</v>
       </c>
       <c r="G6" s="61">
-        <f>IF(OR(D6=0,F6=0),IF(F6=0,0,CEILING(C6/F6,1)),IFERROR(-NPER(D6/100/12,-F6,C6),0))</f>
+        <f>IF(OR(D6=0,F6=0),IF(F6=0,0,CEILING(C6/F6,1)),IFERROR(NPER(D6/100/12,-F6,C6),0))</f>
         <v/>
       </c>
       <c r="H6" s="48">
@@ -10467,7 +10469,7 @@
         <v>50</v>
       </c>
       <c r="G7" s="61">
-        <f>IF(OR(D7=0,F7=0),IF(F7=0,0,CEILING(C7/F7,1)),IFERROR(-NPER(D7/100/12,-F7,C7),0))</f>
+        <f>IF(OR(D7=0,F7=0),IF(F7=0,0,CEILING(C7/F7,1)),IFERROR(NPER(D7/100/12,-F7,C7),0))</f>
         <v/>
       </c>
       <c r="H7" s="48">
@@ -10480,98 +10482,140 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr"/>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
+      <c r="A8" s="35" t="n"/>
+      <c r="B8" s="63" t="n"/>
+      <c r="C8" s="63" t="n"/>
+      <c r="D8" s="64" t="n"/>
+      <c r="E8" s="63" t="n"/>
+      <c r="F8" s="63" t="n"/>
+      <c r="G8" s="61">
+        <f>IF(OR(D8=0,F8=0),IF(F8=0,0,CEILING(C8/F8,1)),IFERROR(NPER(D8/100/12,-F8,C8),0))</f>
+        <v/>
+      </c>
+      <c r="H8" s="48">
+        <f>IFERROR(MAX(0,G8*F8-C8),0)</f>
+        <v/>
+      </c>
       <c r="I8" s="62">
         <f>IF(B8=0,0,MAX(0,(B8-C8)/B8))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr"/>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="A9" s="35" t="n"/>
+      <c r="B9" s="63" t="n"/>
+      <c r="C9" s="63" t="n"/>
+      <c r="D9" s="64" t="n"/>
+      <c r="E9" s="63" t="n"/>
+      <c r="F9" s="63" t="n"/>
+      <c r="G9" s="61">
+        <f>IF(OR(D9=0,F9=0),IF(F9=0,0,CEILING(C9/F9,1)),IFERROR(NPER(D9/100/12,-F9,C9),0))</f>
+        <v/>
+      </c>
+      <c r="H9" s="48">
+        <f>IFERROR(MAX(0,G9*F9-C9),0)</f>
+        <v/>
+      </c>
       <c r="I9" s="62">
         <f>IF(B9=0,0,MAX(0,(B9-C9)/B9))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr"/>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="n"/>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="14" t="n"/>
-      <c r="H10" s="14" t="n"/>
+      <c r="A10" s="35" t="n"/>
+      <c r="B10" s="63" t="n"/>
+      <c r="C10" s="63" t="n"/>
+      <c r="D10" s="64" t="n"/>
+      <c r="E10" s="63" t="n"/>
+      <c r="F10" s="63" t="n"/>
+      <c r="G10" s="61">
+        <f>IF(OR(D10=0,F10=0),IF(F10=0,0,CEILING(C10/F10,1)),IFERROR(NPER(D10/100/12,-F10,C10),0))</f>
+        <v/>
+      </c>
+      <c r="H10" s="48">
+        <f>IFERROR(MAX(0,G10*F10-C10),0)</f>
+        <v/>
+      </c>
       <c r="I10" s="62">
         <f>IF(B10=0,0,MAX(0,(B10-C10)/B10))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr"/>
-      <c r="B11" s="20" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="20" t="n"/>
-      <c r="G11" s="14" t="n"/>
-      <c r="H11" s="14" t="n"/>
+      <c r="A11" s="35" t="n"/>
+      <c r="B11" s="63" t="n"/>
+      <c r="C11" s="63" t="n"/>
+      <c r="D11" s="64" t="n"/>
+      <c r="E11" s="63" t="n"/>
+      <c r="F11" s="63" t="n"/>
+      <c r="G11" s="61">
+        <f>IF(OR(D11=0,F11=0),IF(F11=0,0,CEILING(C11/F11,1)),IFERROR(NPER(D11/100/12,-F11,C11),0))</f>
+        <v/>
+      </c>
+      <c r="H11" s="48">
+        <f>IFERROR(MAX(0,G11*F11-C11),0)</f>
+        <v/>
+      </c>
       <c r="I11" s="62">
         <f>IF(B11=0,0,MAX(0,(B11-C11)/B11))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr"/>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="14" t="n"/>
-      <c r="H12" s="14" t="n"/>
+      <c r="A12" s="35" t="n"/>
+      <c r="B12" s="63" t="n"/>
+      <c r="C12" s="63" t="n"/>
+      <c r="D12" s="64" t="n"/>
+      <c r="E12" s="63" t="n"/>
+      <c r="F12" s="63" t="n"/>
+      <c r="G12" s="61">
+        <f>IF(OR(D12=0,F12=0),IF(F12=0,0,CEILING(C12/F12,1)),IFERROR(NPER(D12/100/12,-F12,C12),0))</f>
+        <v/>
+      </c>
+      <c r="H12" s="48">
+        <f>IFERROR(MAX(0,G12*F12-C12),0)</f>
+        <v/>
+      </c>
       <c r="I12" s="62">
         <f>IF(B12=0,0,MAX(0,(B12-C12)/B12))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr"/>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="n"/>
+      <c r="A13" s="35" t="n"/>
+      <c r="B13" s="63" t="n"/>
+      <c r="C13" s="63" t="n"/>
+      <c r="D13" s="64" t="n"/>
+      <c r="E13" s="63" t="n"/>
+      <c r="F13" s="63" t="n"/>
+      <c r="G13" s="61">
+        <f>IF(OR(D13=0,F13=0),IF(F13=0,0,CEILING(C13/F13,1)),IFERROR(NPER(D13/100/12,-F13,C13),0))</f>
+        <v/>
+      </c>
+      <c r="H13" s="48">
+        <f>IFERROR(MAX(0,G13*F13-C13),0)</f>
+        <v/>
+      </c>
       <c r="I13" s="62">
         <f>IF(B13=0,0,MAX(0,(B13-C13)/B13))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr"/>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="20" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="20" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="14" t="n"/>
+      <c r="A14" s="35" t="n"/>
+      <c r="B14" s="63" t="n"/>
+      <c r="C14" s="63" t="n"/>
+      <c r="D14" s="64" t="n"/>
+      <c r="E14" s="63" t="n"/>
+      <c r="F14" s="63" t="n"/>
+      <c r="G14" s="61">
+        <f>IF(OR(D14=0,F14=0),IF(F14=0,0,CEILING(C14/F14,1)),IFERROR(NPER(D14/100/12,-F14,C14),0))</f>
+        <v/>
+      </c>
+      <c r="H14" s="48">
+        <f>IFERROR(MAX(0,G14*F14-C14),0)</f>
+        <v/>
+      </c>
       <c r="I14" s="62">
         <f>IF(B14=0,0,MAX(0,(B14-C14)/B14))</f>
         <v/>
@@ -11470,12 +11514,12 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="63" t="inlineStr">
+      <c r="A32" s="65" t="inlineStr">
         <is>
           <t>NET WORTH</t>
         </is>
       </c>
-      <c r="B32" s="64">
+      <c r="B32" s="66">
         <f>B15-B30</f>
         <v/>
       </c>
@@ -12774,7 +12818,7 @@
         <f>SUM(M3:M22)</f>
         <v/>
       </c>
-      <c r="N23" s="65">
+      <c r="N23" s="67">
         <f>SUM(N3:N22)</f>
         <v/>
       </c>
@@ -12860,7 +12904,7 @@
         <f>B3-C3</f>
         <v/>
       </c>
-      <c r="E3" s="66">
+      <c r="E3" s="68">
         <f>IF(SUM(C3:C24)=0,0,C3/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -12883,7 +12927,7 @@
         <f>B4-C4</f>
         <v/>
       </c>
-      <c r="E4" s="66">
+      <c r="E4" s="68">
         <f>IF(SUM(C3:C24)=0,0,C4/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -12906,7 +12950,7 @@
         <f>B5-C5</f>
         <v/>
       </c>
-      <c r="E5" s="66">
+      <c r="E5" s="68">
         <f>IF(SUM(C3:C24)=0,0,C5/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -12929,7 +12973,7 @@
         <f>B6-C6</f>
         <v/>
       </c>
-      <c r="E6" s="66">
+      <c r="E6" s="68">
         <f>IF(SUM(C3:C24)=0,0,C6/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -12952,7 +12996,7 @@
         <f>B7-C7</f>
         <v/>
       </c>
-      <c r="E7" s="66">
+      <c r="E7" s="68">
         <f>IF(SUM(C3:C24)=0,0,C7/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -12975,7 +13019,7 @@
         <f>B8-C8</f>
         <v/>
       </c>
-      <c r="E8" s="66">
+      <c r="E8" s="68">
         <f>IF(SUM(C3:C24)=0,0,C8/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -12998,7 +13042,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="66">
+      <c r="E9" s="68">
         <f>IF(SUM(C3:C24)=0,0,C9/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13021,7 +13065,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="66">
+      <c r="E10" s="68">
         <f>IF(SUM(C3:C24)=0,0,C10/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13044,7 +13088,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="66">
+      <c r="E11" s="68">
         <f>IF(SUM(C3:C24)=0,0,C11/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13067,7 +13111,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="66">
+      <c r="E12" s="68">
         <f>IF(SUM(C3:C24)=0,0,C12/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13090,7 +13134,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="66">
+      <c r="E13" s="68">
         <f>IF(SUM(C3:C24)=0,0,C13/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13113,7 +13157,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="66">
+      <c r="E14" s="68">
         <f>IF(SUM(C3:C24)=0,0,C14/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13136,7 +13180,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="66">
+      <c r="E15" s="68">
         <f>IF(SUM(C3:C24)=0,0,C15/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13159,7 +13203,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="66">
+      <c r="E16" s="68">
         <f>IF(SUM(C3:C24)=0,0,C16/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13182,7 +13226,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="66">
+      <c r="E17" s="68">
         <f>IF(SUM(C3:C24)=0,0,C17/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13205,7 +13249,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="66">
+      <c r="E18" s="68">
         <f>IF(SUM(C3:C24)=0,0,C18/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13228,7 +13272,7 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="66">
+      <c r="E19" s="68">
         <f>IF(SUM(C3:C24)=0,0,C19/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13251,7 +13295,7 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="66">
+      <c r="E20" s="68">
         <f>IF(SUM(C3:C24)=0,0,C20/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13274,7 +13318,7 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="66">
+      <c r="E21" s="68">
         <f>IF(SUM(C3:C24)=0,0,C21/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13297,7 +13341,7 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="66">
+      <c r="E22" s="68">
         <f>IF(SUM(C3:C24)=0,0,C22/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13320,7 +13364,7 @@
         <f>B23-C23</f>
         <v/>
       </c>
-      <c r="E23" s="66">
+      <c r="E23" s="68">
         <f>IF(SUM(C3:C24)=0,0,C23/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13343,7 +13387,7 @@
         <f>B24-C24</f>
         <v/>
       </c>
-      <c r="E24" s="66">
+      <c r="E24" s="68">
         <f>IF(SUM(C3:C24)=0,0,C24/SUM(C$3:C$24))</f>
         <v/>
       </c>
@@ -13455,25 +13499,25 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="67" t="n">
+      <c r="A5" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="67" t="n">
+      <c r="B5" s="69" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="67" t="n">
+      <c r="C5" s="69" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="67" t="n">
+      <c r="D5" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="67" t="n">
+      <c r="E5" s="69" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="67" t="n">
+      <c r="F5" s="69" t="n">
         <v>6</v>
       </c>
-      <c r="G5" s="67" t="n">
+      <c r="G5" s="69" t="n">
         <v>7</v>
       </c>
       <c r="J5" s="57">
@@ -13506,25 +13550,25 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="67" t="n">
+      <c r="A6" s="69" t="n">
         <v>8</v>
       </c>
-      <c r="B6" s="67" t="n">
+      <c r="B6" s="69" t="n">
         <v>9</v>
       </c>
-      <c r="C6" s="67" t="n">
+      <c r="C6" s="69" t="n">
         <v>10</v>
       </c>
-      <c r="D6" s="67" t="n">
+      <c r="D6" s="69" t="n">
         <v>11</v>
       </c>
-      <c r="E6" s="67" t="n">
+      <c r="E6" s="69" t="n">
         <v>12</v>
       </c>
-      <c r="F6" s="67" t="n">
+      <c r="F6" s="69" t="n">
         <v>13</v>
       </c>
-      <c r="G6" s="67" t="n">
+      <c r="G6" s="69" t="n">
         <v>14</v>
       </c>
       <c r="J6" s="57">
@@ -13557,25 +13601,25 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="67" t="n">
+      <c r="A7" s="69" t="n">
         <v>15</v>
       </c>
-      <c r="B7" s="67" t="n">
+      <c r="B7" s="69" t="n">
         <v>16</v>
       </c>
-      <c r="C7" s="67" t="n">
+      <c r="C7" s="69" t="n">
         <v>17</v>
       </c>
-      <c r="D7" s="67" t="n">
+      <c r="D7" s="69" t="n">
         <v>18</v>
       </c>
-      <c r="E7" s="67" t="n">
+      <c r="E7" s="69" t="n">
         <v>19</v>
       </c>
-      <c r="F7" s="67" t="n">
+      <c r="F7" s="69" t="n">
         <v>20</v>
       </c>
-      <c r="G7" s="67" t="n">
+      <c r="G7" s="69" t="n">
         <v>21</v>
       </c>
       <c r="J7" s="57">
@@ -13608,25 +13652,25 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="67" t="n">
+      <c r="A8" s="69" t="n">
         <v>22</v>
       </c>
-      <c r="B8" s="67" t="n">
+      <c r="B8" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="C8" s="67" t="n">
+      <c r="C8" s="69" t="n">
         <v>24</v>
       </c>
-      <c r="D8" s="67" t="n">
+      <c r="D8" s="69" t="n">
         <v>25</v>
       </c>
-      <c r="E8" s="67" t="n">
+      <c r="E8" s="69" t="n">
         <v>26</v>
       </c>
-      <c r="F8" s="67" t="n">
+      <c r="F8" s="69" t="n">
         <v>27</v>
       </c>
-      <c r="G8" s="67" t="n">
+      <c r="G8" s="69" t="n">
         <v>28</v>
       </c>
       <c r="J8" s="57">
@@ -13659,13 +13703,13 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="67" t="n">
+      <c r="A9" s="69" t="n">
         <v>29</v>
       </c>
-      <c r="B9" s="67" t="n">
+      <c r="B9" s="69" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="67" t="n">
+      <c r="C9" s="69" t="n">
         <v>31</v>
       </c>
       <c r="J9" s="57">
@@ -13688,7 +13732,7 @@
           <t>No-Spend Days:</t>
         </is>
       </c>
-      <c r="B12" s="68">
+      <c r="B12" s="70">
         <f>IFERROR(COUNTIF(J5:P10,0)-COUNTIF(J5:P10,""),0)</f>
         <v/>
       </c>
@@ -15935,7 +15979,7 @@
           <t>Salary</t>
         </is>
       </c>
-      <c r="B35" s="69" t="inlineStr">
+      <c r="B35" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -15988,7 +16032,7 @@
         <f>IFERROR(VLOOKUP(A35,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O35" s="70">
+      <c r="O35" s="72">
         <f>IFERROR(VLOOKUP(A35,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -15999,7 +16043,7 @@
           <t>Partner Income</t>
         </is>
       </c>
-      <c r="B36" s="69" t="inlineStr">
+      <c r="B36" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16052,7 +16096,7 @@
         <f>IFERROR(VLOOKUP(A36,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O36" s="70">
+      <c r="O36" s="72">
         <f>IFERROR(VLOOKUP(A36,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16063,7 +16107,7 @@
           <t>Freelance</t>
         </is>
       </c>
-      <c r="B37" s="69" t="inlineStr">
+      <c r="B37" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16116,7 +16160,7 @@
         <f>IFERROR(VLOOKUP(A37,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O37" s="70">
+      <c r="O37" s="72">
         <f>IFERROR(VLOOKUP(A37,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16127,7 +16171,7 @@
           <t>Business</t>
         </is>
       </c>
-      <c r="B38" s="69" t="inlineStr">
+      <c r="B38" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16180,7 +16224,7 @@
         <f>IFERROR(VLOOKUP(A38,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O38" s="70">
+      <c r="O38" s="72">
         <f>IFERROR(VLOOKUP(A38,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16191,7 +16235,7 @@
           <t>Investments</t>
         </is>
       </c>
-      <c r="B39" s="69" t="inlineStr">
+      <c r="B39" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16244,7 +16288,7 @@
         <f>IFERROR(VLOOKUP(A39,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O39" s="70">
+      <c r="O39" s="72">
         <f>IFERROR(VLOOKUP(A39,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16255,7 +16299,7 @@
           <t>Rental Income</t>
         </is>
       </c>
-      <c r="B40" s="69" t="inlineStr">
+      <c r="B40" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16308,7 +16352,7 @@
         <f>IFERROR(VLOOKUP(A40,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O40" s="70">
+      <c r="O40" s="72">
         <f>IFERROR(VLOOKUP(A40,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16319,7 +16363,7 @@
           <t>Refunds</t>
         </is>
       </c>
-      <c r="B41" s="69" t="inlineStr">
+      <c r="B41" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16372,7 +16416,7 @@
         <f>IFERROR(VLOOKUP(A41,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O41" s="70">
+      <c r="O41" s="72">
         <f>IFERROR(VLOOKUP(A41,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16383,7 +16427,7 @@
           <t>Other Income</t>
         </is>
       </c>
-      <c r="B42" s="69" t="inlineStr">
+      <c r="B42" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16436,7 +16480,7 @@
         <f>IFERROR(VLOOKUP(A42,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O42" s="70">
+      <c r="O42" s="72">
         <f>IFERROR(VLOOKUP(A42,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16447,7 +16491,7 @@
           <t>Rent/Mortgage</t>
         </is>
       </c>
-      <c r="B43" s="69" t="inlineStr">
+      <c r="B43" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16500,7 +16544,7 @@
         <f>IFERROR(VLOOKUP(A43,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O43" s="70">
+      <c r="O43" s="72">
         <f>IFERROR(VLOOKUP(A43,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16511,7 +16555,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B44" s="69" t="inlineStr">
+      <c r="B44" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16564,7 +16608,7 @@
         <f>IFERROR(VLOOKUP(A44,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O44" s="70">
+      <c r="O44" s="72">
         <f>IFERROR(VLOOKUP(A44,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16575,7 +16619,7 @@
           <t>Groceries</t>
         </is>
       </c>
-      <c r="B45" s="69" t="inlineStr">
+      <c r="B45" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16628,7 +16672,7 @@
         <f>IFERROR(VLOOKUP(A45,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O45" s="70">
+      <c r="O45" s="72">
         <f>IFERROR(VLOOKUP(A45,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16639,7 +16683,7 @@
           <t>Dining Out</t>
         </is>
       </c>
-      <c r="B46" s="69" t="inlineStr">
+      <c r="B46" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16692,7 +16736,7 @@
         <f>IFERROR(VLOOKUP(A46,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O46" s="70">
+      <c r="O46" s="72">
         <f>IFERROR(VLOOKUP(A46,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16703,7 +16747,7 @@
           <t>Transport</t>
         </is>
       </c>
-      <c r="B47" s="69" t="inlineStr">
+      <c r="B47" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16756,7 +16800,7 @@
         <f>IFERROR(VLOOKUP(A47,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O47" s="70">
+      <c r="O47" s="72">
         <f>IFERROR(VLOOKUP(A47,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16767,7 +16811,7 @@
           <t>Fuel</t>
         </is>
       </c>
-      <c r="B48" s="69" t="inlineStr">
+      <c r="B48" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16820,7 +16864,7 @@
         <f>IFERROR(VLOOKUP(A48,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O48" s="70">
+      <c r="O48" s="72">
         <f>IFERROR(VLOOKUP(A48,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16831,7 +16875,7 @@
           <t>Car/Auto</t>
         </is>
       </c>
-      <c r="B49" s="69" t="inlineStr">
+      <c r="B49" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16884,7 +16928,7 @@
         <f>IFERROR(VLOOKUP(A49,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O49" s="70">
+      <c r="O49" s="72">
         <f>IFERROR(VLOOKUP(A49,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16895,7 +16939,7 @@
           <t>Insurance</t>
         </is>
       </c>
-      <c r="B50" s="69" t="inlineStr">
+      <c r="B50" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -16948,7 +16992,7 @@
         <f>IFERROR(VLOOKUP(A50,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O50" s="70">
+      <c r="O50" s="72">
         <f>IFERROR(VLOOKUP(A50,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -16959,7 +17003,7 @@
           <t>Health</t>
         </is>
       </c>
-      <c r="B51" s="69" t="inlineStr">
+      <c r="B51" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17012,7 +17056,7 @@
         <f>IFERROR(VLOOKUP(A51,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O51" s="70">
+      <c r="O51" s="72">
         <f>IFERROR(VLOOKUP(A51,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17023,7 +17067,7 @@
           <t>Phone</t>
         </is>
       </c>
-      <c r="B52" s="69" t="inlineStr">
+      <c r="B52" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17076,7 +17120,7 @@
         <f>IFERROR(VLOOKUP(A52,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O52" s="70">
+      <c r="O52" s="72">
         <f>IFERROR(VLOOKUP(A52,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17087,7 +17131,7 @@
           <t>Internet</t>
         </is>
       </c>
-      <c r="B53" s="69" t="inlineStr">
+      <c r="B53" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17140,7 +17184,7 @@
         <f>IFERROR(VLOOKUP(A53,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O53" s="70">
+      <c r="O53" s="72">
         <f>IFERROR(VLOOKUP(A53,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17151,7 +17195,7 @@
           <t>Subscriptions</t>
         </is>
       </c>
-      <c r="B54" s="69" t="inlineStr">
+      <c r="B54" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17204,7 +17248,7 @@
         <f>IFERROR(VLOOKUP(A54,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O54" s="70">
+      <c r="O54" s="72">
         <f>IFERROR(VLOOKUP(A54,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17215,7 +17259,7 @@
           <t>Entertainment</t>
         </is>
       </c>
-      <c r="B55" s="69" t="inlineStr">
+      <c r="B55" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17268,7 +17312,7 @@
         <f>IFERROR(VLOOKUP(A55,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O55" s="70">
+      <c r="O55" s="72">
         <f>IFERROR(VLOOKUP(A55,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17279,7 +17323,7 @@
           <t>Shopping</t>
         </is>
       </c>
-      <c r="B56" s="69" t="inlineStr">
+      <c r="B56" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17332,7 +17376,7 @@
         <f>IFERROR(VLOOKUP(A56,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O56" s="70">
+      <c r="O56" s="72">
         <f>IFERROR(VLOOKUP(A56,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17343,7 +17387,7 @@
           <t>Clothing</t>
         </is>
       </c>
-      <c r="B57" s="69" t="inlineStr">
+      <c r="B57" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17396,7 +17440,7 @@
         <f>IFERROR(VLOOKUP(A57,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O57" s="70">
+      <c r="O57" s="72">
         <f>IFERROR(VLOOKUP(A57,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17407,7 +17451,7 @@
           <t>Personal Care</t>
         </is>
       </c>
-      <c r="B58" s="69" t="inlineStr">
+      <c r="B58" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17460,7 +17504,7 @@
         <f>IFERROR(VLOOKUP(A58,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O58" s="70">
+      <c r="O58" s="72">
         <f>IFERROR(VLOOKUP(A58,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17471,7 +17515,7 @@
           <t>Gym/Fitness</t>
         </is>
       </c>
-      <c r="B59" s="69" t="inlineStr">
+      <c r="B59" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17524,7 +17568,7 @@
         <f>IFERROR(VLOOKUP(A59,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O59" s="70">
+      <c r="O59" s="72">
         <f>IFERROR(VLOOKUP(A59,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17535,7 +17579,7 @@
           <t>Pets</t>
         </is>
       </c>
-      <c r="B60" s="69" t="inlineStr">
+      <c r="B60" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17588,7 +17632,7 @@
         <f>IFERROR(VLOOKUP(A60,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O60" s="70">
+      <c r="O60" s="72">
         <f>IFERROR(VLOOKUP(A60,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17599,7 +17643,7 @@
           <t>Kids</t>
         </is>
       </c>
-      <c r="B61" s="69" t="inlineStr">
+      <c r="B61" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17652,7 +17696,7 @@
         <f>IFERROR(VLOOKUP(A61,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O61" s="70">
+      <c r="O61" s="72">
         <f>IFERROR(VLOOKUP(A61,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17663,7 +17707,7 @@
           <t>Gifts/Donations</t>
         </is>
       </c>
-      <c r="B62" s="69" t="inlineStr">
+      <c r="B62" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17716,7 +17760,7 @@
         <f>IFERROR(VLOOKUP(A62,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O62" s="70">
+      <c r="O62" s="72">
         <f>IFERROR(VLOOKUP(A62,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17727,7 +17771,7 @@
           <t>Travel</t>
         </is>
       </c>
-      <c r="B63" s="69" t="inlineStr">
+      <c r="B63" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17780,7 +17824,7 @@
         <f>IFERROR(VLOOKUP(A63,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O63" s="70">
+      <c r="O63" s="72">
         <f>IFERROR(VLOOKUP(A63,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>
@@ -17791,7 +17835,7 @@
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B64" s="69" t="inlineStr">
+      <c r="B64" s="71" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
@@ -17844,7 +17888,7 @@
         <f>IFERROR(VLOOKUP(A64,Settings!$A$30:$C$59,3,FALSE),0)</f>
         <v/>
       </c>
-      <c r="O64" s="70">
+      <c r="O64" s="72">
         <f>IFERROR(VLOOKUP(A64,Settings!$A$30:$C$59,3,FALSE),0)*12</f>
         <v/>
       </c>

</xml_diff>